<commit_message>
updated template and config.json to reflect the new nullable asu-group field
</commit_message>
<xml_diff>
--- a/models/anse-template.xlsx
+++ b/models/anse-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shxie/projects/anse-models/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shxie/projects/anse-public-releases/models/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BFE4496-70F5-3E4B-ADF9-0F5FE5EC87BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B01BFF7A-44C2-764C-9605-355C9292E770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20640" yWindow="3840" windowWidth="29580" windowHeight="20860" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9600" yWindow="4500" windowWidth="35260" windowHeight="20860" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs - Flow Network" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,6 @@
     <author>tc={00BD00F7-005E-4DB0-8E4F-00F100D200FB}</author>
     <author>tc={0090004E-00C8-46F8-AD59-009500D200CE}</author>
     <author>tc={001E0064-0036-4F2D-AF39-003100B800F7}</author>
-    <author>tc={00EE009D-0041-4A9F-9B16-00EC0037006E}</author>
     <author>tc={003C0055-0015-41D7-BFA4-000E00920078}</author>
     <author>tc={005600D5-0083-4DBD-AA08-009B00FD00AD}</author>
     <author>tc={0010001E-00BA-4128-B0F1-00EF00D50023}</author>
@@ -144,16 +143,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="E12" authorId="11" shapeId="0" xr:uid="{00EE009D-0041-4A9F-9B16-00EC0037006E}">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    If unknown, enter "UNIVERSE"
-</t>
-      </text>
-    </comment>
-    <comment ref="F12" authorId="12" shapeId="0" xr:uid="{003C0055-0015-41D7-BFA4-000E00920078}">
+    <comment ref="F12" authorId="11" shapeId="0" xr:uid="{003C0055-0015-41D7-BFA4-000E00920078}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -162,7 +152,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="G12" authorId="13" shapeId="0" xr:uid="{005600D5-0083-4DBD-AA08-009B00FD00AD}">
+    <comment ref="G12" authorId="12" shapeId="0" xr:uid="{005600D5-0083-4DBD-AA08-009B00FD00AD}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -171,7 +161,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="D15" authorId="14" shapeId="0" xr:uid="{0010001E-00BA-4128-B0F1-00EF00D50023}">
+    <comment ref="D15" authorId="13" shapeId="0" xr:uid="{0010001E-00BA-4128-B0F1-00EF00D50023}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -180,7 +170,7 @@
 </t>
       </text>
     </comment>
-    <comment ref="G15" authorId="15" shapeId="0" xr:uid="{06ADED73-FE3A-AB44-9B8D-57BD030E94DF}">
+    <comment ref="G15" authorId="14" shapeId="0" xr:uid="{06ADED73-FE3A-AB44-9B8D-57BD030E94DF}">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -572,12 +562,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -866,10 +857,6 @@
     <text xml:space="preserve">If unknown, enter name of the EVENT for which the ACTION_PARAMETER_SET will be relevant
 </text>
   </threadedComment>
-  <threadedComment ref="E12" personId="{3B3DA95D-9B14-85C2-BBBD-4F6E774A6498}" id="{00EE009D-0041-4A9F-9B16-00EC0037006E}">
-    <text xml:space="preserve">If unknown, enter "UNIVERSE"
-</text>
-  </threadedComment>
   <threadedComment ref="F12" personId="{3B3DA95D-9B14-85C2-BBBD-4F6E774A6498}" id="{003C0055-0015-41D7-BFA4-000E00920078}">
     <text xml:space="preserve">Integer field
 </text>
@@ -1050,7 +1037,7 @@
       <c r="D12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F12" s="1" t="s">
@@ -1407,7 +1394,7 @@
       <c r="D5" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="5" t="s">
         <v>18</v>
       </c>
       <c r="F5" s="2" t="s">

</xml_diff>